<commit_message>
feat: Add AnexoProyectos and AnexoGrupos templates with corresponding sheets
- Implemented AnexoProyectos template with multiple sheets for different project types (PAPN, PAPS, PAPT, PE, PNE, PDL, PRCI, PNAP, Nuevas Aplicaciones).
- Created AnexoGruposTemplate and GruposSheet for generating group research data.
- Defined headers and template cells for each sheet to facilitate data entry.
- Set up styling and formatting for Excel output using ClosedXML.
</commit_message>
<xml_diff>
--- a/Dashboard_v2/src/Infrastructure/Templates/AnexoGrupos.xlsx
+++ b/Dashboard_v2/src/Infrastructure/Templates/AnexoGrupos.xlsx
@@ -21,124 +21,124 @@
     <x:t>GRUPOS DE INVESTIGACIÓN</x:t>
   </x:si>
   <x:si>
+    <x:t>Nombre del Grupo de Investigación</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Total de Integrantes</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Áreas de la UH de sus Miembros</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Dr</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MSc</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Lic</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PAUX</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PASIST</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INST</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IAUX</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IAGRG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ASP.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Adiestrados</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Técnicos / Especialistas</x:t>
+  </x:si>
+  <x:si>
+    <x:t>No Estudiantes 1ro-2do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>No Estudiantes 3ro-4to</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Área Temática UH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Línea de Investigación</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Proyectos de Investigación del Grupo *</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.Nombre}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.TotalIntegrantes}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.CantDoctores}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.CantMasters}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.CantLicenciados}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.CantPT}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.CantPAUX}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.CantPASIST}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.CantINST}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.CantIT}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.CantIAUX}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.CantIAGRG}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.CantASP}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.CantAdiestrados}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.AreaTematica}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.LineasDeInvestigacion}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
     <x:t>* código y título del proyecto</x:t>
   </x:si>
   <x:si>
     <x:t>** si el grupo es ejecutor principal</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Nombre del Grupo de Investigación</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Total de Integrantes</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Áreas de la UH de sus Miembros</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Dr</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MSc</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Lic</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PAUX</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PASIST</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INST</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IAUX</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IAGRG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ASP.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Adiestrados</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Técnicos / Especialistas</x:t>
-  </x:si>
-  <x:si>
-    <x:t>No Estudiantes 1ro-2do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>No Estudiantes 3ro-4to</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Área Temática UH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Línea de Investigación</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Proyectos de Investigación del Grupo *</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.Nombre}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.TotalIntegrantes}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.CantDoctores}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.CantMasters}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.CantLicenciados}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.CantPT}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.CantPAUX}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.CantPASIST}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.CantINST}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.CantIT}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.CantIAUX}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.CantIAGRG}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.CantASP}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.CantAdiestrados}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.AreaTematica}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{item.LineasDeInvestigacion}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
   </x:si>
 </x:sst>
 </file>
@@ -270,11 +270,11 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellXfs>
@@ -591,137 +591,147 @@
     </x:row>
     <x:row r="2" spans="1:23">
       <x:c r="W2" s="2" t="s">
-        <x:v>1</x:v>
+        <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:23">
       <x:c r="W3" s="2" t="s">
-        <x:v>2</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:23" ht="50" customHeight="1">
       <x:c r="A4" s="3" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C4" s="3" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="s">
+      <x:c r="D4" s="3" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C4" s="3" t="s">
+      <x:c r="E4" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D4" s="3" t="s">
+      <x:c r="F4" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="E4" s="3" t="s">
+      <x:c r="G4" s="3" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="F4" s="3" t="s">
+      <x:c r="H4" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="G4" s="3" t="s">
+      <x:c r="I4" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="H4" s="3" t="s">
+      <x:c r="J4" s="3" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="I4" s="3" t="s">
+      <x:c r="K4" s="3" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="J4" s="3" t="s">
+      <x:c r="L4" s="3" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="K4" s="3" t="s">
+      <x:c r="M4" s="3" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="L4" s="3" t="s">
+      <x:c r="N4" s="3" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="M4" s="3" t="s">
+      <x:c r="O4" s="3" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="N4" s="3" t="s">
+      <x:c r="P4" s="3" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="O4" s="3" t="s">
+      <x:c r="Q4" s="3" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="P4" s="3" t="s">
+      <x:c r="R4" s="3" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="Q4" s="3" t="s">
+      <x:c r="S4" s="3" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="R4" s="3" t="s">
+      <x:c r="T4" s="3" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="S4" s="3" t="s">
+      <x:c r="U4" s="3" t="s">
         <x:v>21</x:v>
-      </x:c>
-      <x:c r="T4" s="3" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="U4" s="3" t="s">
-        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:23">
       <x:c r="A5" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C5" s="5" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="s">
+      <x:c r="E5" s="4" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="C5" s="4"/>
-      <x:c r="D5" s="5" t="s">
+      <x:c r="F5" s="4" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="E5" s="5" t="s">
+      <x:c r="G5" s="4" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="F5" s="5" t="s">
+      <x:c r="H5" s="4" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="G5" s="5" t="s">
+      <x:c r="I5" s="4" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="H5" s="5" t="s">
+      <x:c r="J5" s="4" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="I5" s="5" t="s">
+      <x:c r="K5" s="4" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="J5" s="5" t="s">
+      <x:c r="L5" s="4" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="K5" s="5" t="s">
+      <x:c r="M5" s="4" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="L5" s="5" t="s">
+      <x:c r="N5" s="4" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="M5" s="5" t="s">
+      <x:c r="O5" s="4" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="N5" s="5" t="s">
+      <x:c r="P5" s="5" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="Q5" s="5" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="R5" s="5" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="S5" s="4" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="O5" s="5" t="s">
+      <x:c r="T5" s="4" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="P5" s="4"/>
-      <x:c r="Q5" s="4"/>
-      <x:c r="R5" s="4"/>
-      <x:c r="S5" s="4" t="s">
+      <x:c r="U5" s="5" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="T5" s="4" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="U5" s="4"/>
     </x:row>
     <x:row r="6" spans="1:23">
       <x:c r="A6" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>